<commit_message>
feature: change in prediction value to sum region means instead or averaging them
</commit_message>
<xml_diff>
--- a/checkpoint_robuspredictor.xlsx
+++ b/checkpoint_robuspredictor.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:AA9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,77 +448,122 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>suma_promedios_region</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>promedio_promedios_region</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>promedios_region_por_dominio</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>motivo_rechazo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>profundidad_particion</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>var1</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>var2</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>var3</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>datos_entrenamiento</t>
+          <t>prom_var1_dom1</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>target_entrenamiento</t>
+          <t>prom_var1_dom2</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>cantidad_entrenamiento</t>
+          <t>prom_var1_consol</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>promedio_entrenamiento</t>
+          <t>prom_var2_dom1</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>desviacion_entrenamiento</t>
+          <t>prom_var2_dom2</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>datos_validacion</t>
+          <t>prom_var2_consol</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>target_validacion</t>
+          <t>prom_var3_dom1</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>cantidad_validacion</t>
+          <t>prom_var3_dom2</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>promedio_validacion</t>
+          <t>prom_var3_consol</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>desviacion_validacion</t>
+          <t>n_dom1</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>prom_target_dom1</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>std_target_dom1</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>n_dom2</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>prom_target_dom2</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>std_target_dom2</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>n_testing</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>prom_target_testing</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>std_target_testing</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>prom_target_consolidado</t>
         </is>
       </c>
     </row>
@@ -532,74 +577,77 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E2" t="n">
         <v>1.535</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>[1.55, 1.52]</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="H2" t="n">
         <v>3</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10.0 - 11.0</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>20.0 - 21.0</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>30.0 - 31.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>[{"indice": 1, "var1": 10.0, "var2": 20.0, "var3": 30.0}, {"indice": 4, "var1": 11.0, "var2": 21.0, "var3": 31.0}]</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>[{"indice": 1, "valor": 1.5}, {"indice": 4, "valor": 1.6}]</t>
-        </is>
+      <c r="I2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>10.5</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>10.5</v>
       </c>
       <c r="L2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="M2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="N2" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="O2" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="P2" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
         <v>1.55</v>
       </c>
-      <c r="M2" t="n">
-        <v>0.07071067811865482</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 20, "var1": 10.5, "var2": 20.5, "var3": 30.5}]}]</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 20, "valor": 1.52}]}]</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 1}]</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 1.52}]</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.0}]</t>
-        </is>
+      <c r="T2" t="n">
+        <v>0.070711</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V2" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="n">
+        <v>1.535</v>
       </c>
     </row>
     <row r="3">
@@ -612,74 +660,77 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
+        <v>3.195</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.195</v>
+      </c>
+      <c r="E3" t="n">
         <v>1.5975</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>[1.6, 1.5950000000000002]</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="H3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>12.0 - 13.0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>22.0 - 23.0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>32.0 - 33.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>[{"indice": 6, "var1": 12.0, "var2": 22.0, "var3": 32.0}, {"indice": 2, "var1": 13.0, "var2": 23.0, "var3": 33.0}]</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>[{"indice": 6, "valor": 1.55}, {"indice": 2, "valor": 1.65}]</t>
-        </is>
+      <c r="I3" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="J3" t="n">
+        <v>12</v>
       </c>
       <c r="K3" t="n">
-        <v>2</v>
+        <v>12.25</v>
       </c>
       <c r="L3" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="M3" t="n">
+        <v>22</v>
+      </c>
+      <c r="N3" t="n">
+        <v>22.25</v>
+      </c>
+      <c r="O3" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="P3" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="R3" t="n">
+        <v>2</v>
+      </c>
+      <c r="S3" t="n">
         <v>1.6</v>
       </c>
-      <c r="M3" t="n">
-        <v>0.07071067811865465</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 16, "var1": 12.5, "var2": 22.5, "var3": 32.5}, {"indice": 18, "var1": 11.5, "var2": 21.5, "var3": 31.5}]}]</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 16, "valor": 1.57}, {"indice": 18, "valor": 1.62}]}]</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 2}]</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 1.5950000000000002}]</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.03535533905932741}]</t>
-        </is>
+      <c r="T3" t="n">
+        <v>0.070711</v>
+      </c>
+      <c r="U3" t="n">
+        <v>2</v>
+      </c>
+      <c r="V3" t="n">
+        <v>1.595</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.035355</v>
+      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="n">
+        <v>1.5975</v>
       </c>
     </row>
     <row r="4">
@@ -692,74 +743,77 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="E4" t="n">
         <v>1.6875</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[1.69, 1.685]</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="H4" t="n">
         <v>3</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>14.0 - 15.0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>24.0 - 25.0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>34.0 - 35.0</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>[{"indice": 12, "var1": 14.0, "var2": 24.0, "var3": 34.0}, {"indice": 8, "var1": 15.0, "var2": 25.0, "var3": 35.0}]</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>[{"indice": 12, "valor": 1.68}, {"indice": 8, "valor": 1.7}]</t>
-        </is>
+      <c r="I4" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>14</v>
       </c>
       <c r="K4" t="n">
-        <v>2</v>
+        <v>14.25</v>
       </c>
       <c r="L4" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="M4" t="n">
+        <v>24</v>
+      </c>
+      <c r="N4" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="O4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="P4" t="n">
+        <v>34</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>34.25</v>
+      </c>
+      <c r="R4" t="n">
+        <v>2</v>
+      </c>
+      <c r="S4" t="n">
         <v>1.69</v>
       </c>
-      <c r="M4" t="n">
-        <v>0.01414213562373096</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 22, "var1": 13.5, "var2": 23.5, "var3": 33.5}, {"indice": 28, "var1": 14.5, "var2": 24.5, "var3": 34.5}]}]</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 22, "valor": 1.67}, {"indice": 28, "valor": 1.7}]}]</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 2}]</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 1.685}]</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.021213203435596444}]</t>
-        </is>
+      <c r="T4" t="n">
+        <v>0.014142</v>
+      </c>
+      <c r="U4" t="n">
+        <v>2</v>
+      </c>
+      <c r="V4" t="n">
+        <v>1.685</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.021213</v>
+      </c>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="n">
+        <v>1.6875</v>
       </c>
     </row>
     <row r="5">
@@ -772,74 +826,77 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="E5" t="n">
         <v>1.755</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>[1.7650000000000001, 1.745]</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="H5" t="n">
         <v>3</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>16.0 - 17.0</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>26.0 - 27.0</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>36.0 - 37.0</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>[{"indice": 10, "var1": 16.0, "var2": 26.0, "var3": 36.0}, {"indice": 14, "var1": 17.0, "var2": 27.0, "var3": 37.0}]</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>[{"indice": 10, "valor": 1.75}, {"indice": 14, "valor": 1.78}]</t>
-        </is>
+      <c r="I5" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>16</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>16.25</v>
       </c>
       <c r="L5" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="M5" t="n">
+        <v>26</v>
+      </c>
+      <c r="N5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="O5" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="P5" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>36.25</v>
+      </c>
+      <c r="R5" t="n">
+        <v>2</v>
+      </c>
+      <c r="S5" t="n">
         <v>1.765</v>
       </c>
-      <c r="M5" t="n">
-        <v>0.02121320343559644</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 24, "var1": 15.5, "var2": 25.5, "var3": 35.5}, {"indice": 26, "var1": 16.5, "var2": 26.5, "var3": 36.5}]}]</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 24, "valor": 1.72}, {"indice": 26, "valor": 1.77}]}]</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 2}]</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 1.745}]</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.03535533905932741}]</t>
-        </is>
+      <c r="T5" t="n">
+        <v>0.021213</v>
+      </c>
+      <c r="U5" t="n">
+        <v>2</v>
+      </c>
+      <c r="V5" t="n">
+        <v>1.745</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.035355</v>
+      </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="n">
+        <v>1.755</v>
       </c>
     </row>
     <row r="6">
@@ -852,74 +909,77 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="E6" t="n">
         <v>2.355</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>[2.55, 2.16]</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>["Dominio 2: std fuera de rango: 0.5091168824543142 no está entre 0.0 y 0.5"]</t>
         </is>
       </c>
-      <c r="E6" t="n">
+      <c r="H6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>50.0 - 51.0</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>80.0 - 81.0</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>90.0 - 91.0</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>[{"indice": 5, "var1": 50.0, "var2": 80.0, "var3": 90.0}, {"indice": 3, "var1": 51.0, "var2": 81.0, "var3": 91.0}]</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>[{"indice": 5, "valor": 2.5}, {"indice": 3, "valor": 2.6}]</t>
-        </is>
+      <c r="I6" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>34</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>42.25</v>
       </c>
       <c r="L6" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="M6" t="n">
+        <v>54</v>
+      </c>
+      <c r="N6" t="n">
+        <v>67.25</v>
+      </c>
+      <c r="O6" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="P6" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>77.25</v>
+      </c>
+      <c r="R6" t="n">
+        <v>2</v>
+      </c>
+      <c r="S6" t="n">
         <v>2.55</v>
       </c>
-      <c r="M6" t="n">
-        <v>0.07071067811865482</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 17, "var1": 50.5, "var2": 80.5, "var3": 90.5}, {"indice": 30, "var1": 17.5, "var2": 27.5, "var3": 37.5}]}]</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 17, "valor": 2.52}, {"indice": 30, "valor": 1.8}]}]</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 2}]</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 2.16}]</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.5091168824543142}]</t>
-        </is>
+      <c r="T6" t="n">
+        <v>0.070711</v>
+      </c>
+      <c r="U6" t="n">
+        <v>2</v>
+      </c>
+      <c r="V6" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="W6" t="n">
+        <v>0.509117</v>
+      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="n">
+        <v>2.355</v>
       </c>
     </row>
     <row r="7">
@@ -932,74 +992,77 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
+        <v>5.194999999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.194999999999999</v>
+      </c>
+      <c r="E7" t="n">
         <v>2.5975</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>[2.5999999999999996, 2.5949999999999998]</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E7" t="n">
+      <c r="H7" t="n">
         <v>3</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>52.0 - 53.0</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>82.0 - 83.0</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>92.0 - 93.0</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>[{"indice": 0, "var1": 52.0, "var2": 82.0, "var3": 92.0}, {"indice": 7, "var1": 53.0, "var2": 83.0, "var3": 93.0}]</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>[{"indice": 0, "valor": 2.55}, {"indice": 7, "valor": 2.65}]</t>
-        </is>
+      <c r="I7" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>52</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>52.25</v>
       </c>
       <c r="L7" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="M7" t="n">
+        <v>82</v>
+      </c>
+      <c r="N7" t="n">
+        <v>82.25</v>
+      </c>
+      <c r="O7" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="P7" t="n">
+        <v>92</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>92.25</v>
+      </c>
+      <c r="R7" t="n">
+        <v>2</v>
+      </c>
+      <c r="S7" t="n">
         <v>2.6</v>
       </c>
-      <c r="M7" t="n">
-        <v>0.07071067811865482</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 21, "var1": 52.5, "var2": 82.5, "var3": 92.5}, {"indice": 23, "var1": 51.5, "var2": 81.5, "var3": 91.5}]}]</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 21, "valor": 2.57}, {"indice": 23, "valor": 2.62}]}]</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 2}]</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 2.5949999999999998}]</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.03535533905932756}]</t>
-        </is>
+      <c r="T7" t="n">
+        <v>0.070711</v>
+      </c>
+      <c r="U7" t="n">
+        <v>2</v>
+      </c>
+      <c r="V7" t="n">
+        <v>2.595</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0.035355</v>
+      </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="n">
+        <v>2.5975</v>
       </c>
     </row>
     <row r="8">
@@ -1012,74 +1075,77 @@
         <v>1</v>
       </c>
       <c r="C8" t="n">
+        <v>5.375</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5.375</v>
+      </c>
+      <c r="E8" t="n">
         <v>2.6875</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>[2.6900000000000004, 2.685]</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E8" t="n">
+      <c r="H8" t="n">
         <v>3</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>54.0 - 55.0</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>84.0 - 85.0</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>94.0 - 95.0</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>[{"indice": 13, "var1": 54.0, "var2": 84.0, "var3": 94.0}, {"indice": 9, "var1": 55.0, "var2": 85.0, "var3": 95.0}]</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>[{"indice": 13, "valor": 2.68}, {"indice": 9, "valor": 2.7}]</t>
-        </is>
+      <c r="I8" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>54</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>54.25</v>
       </c>
       <c r="L8" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="M8" t="n">
+        <v>84</v>
+      </c>
+      <c r="N8" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="O8" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="P8" t="n">
+        <v>94</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>94.25</v>
+      </c>
+      <c r="R8" t="n">
+        <v>2</v>
+      </c>
+      <c r="S8" t="n">
         <v>2.69</v>
       </c>
-      <c r="M8" t="n">
-        <v>0.01414213562373096</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 19, "var1": 53.5, "var2": 83.5, "var3": 93.5}, {"indice": 29, "var1": 54.5, "var2": 84.5, "var3": 94.5}]}]</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 19, "valor": 2.67}, {"indice": 29, "valor": 2.7}]}]</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 2}]</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 2.685}]</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.0212132034355966}]</t>
-        </is>
+      <c r="T8" t="n">
+        <v>0.014142</v>
+      </c>
+      <c r="U8" t="n">
+        <v>2</v>
+      </c>
+      <c r="V8" t="n">
+        <v>2.685</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0.021213</v>
+      </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="n">
+        <v>2.6875</v>
       </c>
     </row>
     <row r="9">
@@ -1092,74 +1158,77 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
+        <v>5.528333333333332</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5.528333333333332</v>
+      </c>
+      <c r="E9" t="n">
         <v>2.764166666666666</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>[2.7649999999999997, 2.763333333333333]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="E9" t="n">
+      <c r="H9" t="n">
         <v>3</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>56.0 - 57.0</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>86.0 - 87.0</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>96.0 - 97.0</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>[{"indice": 11, "var1": 56.0, "var2": 86.0, "var3": 96.0}, {"indice": 15, "var1": 57.0, "var2": 87.0, "var3": 97.0}]</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>[{"indice": 11, "valor": 2.75}, {"indice": 15, "valor": 2.78}]</t>
-        </is>
+      <c r="I9" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>56.5</v>
       </c>
       <c r="K9" t="n">
-        <v>2</v>
+        <v>56.5</v>
       </c>
       <c r="L9" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="M9" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="O9" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="P9" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="R9" t="n">
+        <v>2</v>
+      </c>
+      <c r="S9" t="n">
         <v>2.765</v>
       </c>
-      <c r="M9" t="n">
-        <v>0.02121320343559629</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "datos": [{"indice": 25, "var1": 55.5, "var2": 85.5, "var3": 95.5}, {"indice": 27, "var1": 56.5, "var2": 86.5, "var3": 96.5}, {"indice": 31, "var1": 57.5, "var2": 87.5, "var3": 97.5}]}]</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "target": [{"indice": 25, "valor": 2.72}, {"indice": 27, "valor": 2.77}, {"indice": 31, "valor": 2.8}]}]</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "cantidad": 3}]</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "promedio": 2.763333333333333}]</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>[{"dominio": 2, "desviacion": 0.04041451884327362}]</t>
-        </is>
+      <c r="T9" t="n">
+        <v>0.021213</v>
+      </c>
+      <c r="U9" t="n">
+        <v>3</v>
+      </c>
+      <c r="V9" t="n">
+        <v>2.763333</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.040415</v>
+      </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="n">
+        <v>2.764166</v>
       </c>
     </row>
   </sheetData>
@@ -1204,12 +1273,12 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>tamaño_izquierda</t>
+          <t>tamanio_izquierda</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>tamaño_derecha</t>
+          <t>tamanio_derecha</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -1737,7 +1806,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dominio_1_tamaño_minimo_grupo</t>
+          <t>dominio_1_tamanio_minimo_grupo</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1747,7 +1816,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dominio_1_tamaño_maximo_grupo</t>
+          <t>dominio_1_tamanio_maximo_grupo</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1757,7 +1826,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dominio_1_tamaño_promedio_grupo</t>
+          <t>dominio_1_tamanio_promedio_grupo</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1787,7 +1856,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dominio_2_tamaño_minimo_grupo</t>
+          <t>dominio_2_tamanio_minimo_grupo</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1797,7 +1866,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dominio_2_tamaño_maximo_grupo</t>
+          <t>dominio_2_tamanio_maximo_grupo</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1807,7 +1876,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dominio_2_tamaño_promedio_grupo</t>
+          <t>dominio_2_tamanio_promedio_grupo</t>
         </is>
       </c>
       <c r="B17" t="n">

</xml_diff>